<commit_message>
conteneur 3 de vectorisation fonctionnel
</commit_message>
<xml_diff>
--- a/data/opendata/hashFiles.xlsx
+++ b/data/opendata/hashFiles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,6 +437,18 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>2026-05-14 16:34:29.291064</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>58ce0efd3aaa2a713dbc4138eb1329e3</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:22:46.435453</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
conteneur 4 de test de vectorisation fonctionnel
</commit_message>
<xml_diff>
--- a/data/opendata/hashFiles.xlsx
+++ b/data/opendata/hashFiles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,54 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>58ce0efd3aaa2a713dbc4138eb1329e3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-05-16 16:43:44.479683</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>58ce0efd3aaa2a713dbc4138eb1329e3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-05-16 17:00:45.411476</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>58ce0efd3aaa2a713dbc4138eb1329e3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-05-16 17:01:56.145331</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>58ce0efd3aaa2a713dbc4138eb1329e3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-05-16 17:03:07.071900</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
conteneur 05 de récupération des reponses via Mistral fonctionnel
</commit_message>
<xml_diff>
--- a/data/opendata/hashFiles.xlsx
+++ b/data/opendata/hashFiles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,6 +500,18 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1ffc7ca53484e83ec88d9a0903c481ed</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-05-17 10:57:55.917586</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
conteneur 6 de test ragas fonctionnel
</commit_message>
<xml_diff>
--- a/data/opendata/hashFiles.xlsx
+++ b/data/opendata/hashFiles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,6 +512,18 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>6bdfaff65fce99e1451c40021b394d42</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-05-17 11:56:10.294401</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
conteneur 07 chatbot fonctionnel
</commit_message>
<xml_diff>
--- a/data/opendata/hashFiles.xlsx
+++ b/data/opendata/hashFiles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,96 +431,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>9ffe7f6c697cebe52d682105e6ee8751</t>
+          <t>2855e37ac952d181624675dbc0e2b9cd</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-14 16:34:29.291064</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>58ce0efd3aaa2a713dbc4138eb1329e3</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-05-16 14:22:46.435453</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>58ce0efd3aaa2a713dbc4138eb1329e3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-05-16 16:43:44.479683</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>58ce0efd3aaa2a713dbc4138eb1329e3</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-05-16 17:00:45.411476</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>58ce0efd3aaa2a713dbc4138eb1329e3</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-05-16 17:01:56.145331</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>58ce0efd3aaa2a713dbc4138eb1329e3</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-05-16 17:03:07.071900</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1ffc7ca53484e83ec88d9a0903c481ed</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-05-17 10:57:55.917586</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>6bdfaff65fce99e1451c40021b394d42</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-05-17 11:56:10.294401</t>
+          <t>2026-05-17 16:31:33.507958</t>
         </is>
       </c>
     </row>

</xml_diff>